<commit_message>
Update production rangers xlsx with expanded CHPU 2026 roster.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/Рейнджеры_производственная_группа.xlsx
+++ b/data/Рейнджеры_производственная_группа.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="РОБО" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ЧПУ'!$A$1:$M$356</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ЧПУ'!$A$1:$M$354</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'МИКРО'!$A$1:$M$122</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'АЭРО'!$A$1:$M$84</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'РОБО'!$A$1:$M$109</definedName>
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M356"/>
+  <dimension ref="A1:M354"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -16040,66 +16040,8 @@
         </is>
       </c>
     </row>
-    <row r="355">
-      <c r="A355" s="2" t="n">
-        <v>354</v>
-      </c>
-      <c r="B355" s="2" t="inlineStr">
-        <is>
-          <t>ЧПУ (уточнить)</t>
-        </is>
-      </c>
-      <c r="C355" s="2" t="inlineStr">
-        <is>
-          <t>Мелисбеков Нуржан Сыргабекович</t>
-        </is>
-      </c>
-      <c r="D355" s="2" t="inlineStr"/>
-      <c r="E355" s="2" t="inlineStr"/>
-      <c r="F355" s="2" t="inlineStr"/>
-      <c r="G355" s="2" t="inlineStr"/>
-      <c r="H355" s="2" t="inlineStr"/>
-      <c r="I355" s="2" t="inlineStr"/>
-      <c r="J355" s="2" t="inlineStr"/>
-      <c r="K355" s="2" t="inlineStr"/>
-      <c r="L355" s="2" t="inlineStr"/>
-      <c r="M355" s="2" t="inlineStr">
-        <is>
-          <t>учится</t>
-        </is>
-      </c>
-    </row>
-    <row r="356">
-      <c r="A356" s="2" t="n">
-        <v>355</v>
-      </c>
-      <c r="B356" s="2" t="inlineStr">
-        <is>
-          <t>ЧПУ (уточнить)</t>
-        </is>
-      </c>
-      <c r="C356" s="2" t="inlineStr">
-        <is>
-          <t>Морозов Андрей Витальевич</t>
-        </is>
-      </c>
-      <c r="D356" s="2" t="inlineStr"/>
-      <c r="E356" s="2" t="inlineStr"/>
-      <c r="F356" s="2" t="inlineStr"/>
-      <c r="G356" s="2" t="inlineStr"/>
-      <c r="H356" s="2" t="inlineStr"/>
-      <c r="I356" s="2" t="inlineStr"/>
-      <c r="J356" s="2" t="inlineStr"/>
-      <c r="K356" s="2" t="inlineStr"/>
-      <c r="L356" s="2" t="inlineStr"/>
-      <c r="M356" s="2" t="inlineStr">
-        <is>
-          <t>учится</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:M356"/>
+  <autoFilter ref="A1:M354"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>